<commit_message>
Fixed the database, the margins and texts.
</commit_message>
<xml_diff>
--- a/data/GTF BIG Talent Scholars.xlsx
+++ b/data/GTF BIG Talent Scholars.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\s2730428\Documents\GTF\global-talent-map\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\iona.sms.ed.ac.uk\home\s2730428\GTF-Impact-Map\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89D66817-5C70-4BAA-A515-B57ED673FF17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{044BD7FC-82BE-4106-904E-83837A500776}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Global Talent Fund - BIG Schola" sheetId="1" r:id="rId1"/>
@@ -312,9 +312,6 @@
     <t>Australia</t>
   </si>
   <si>
-    <t>Turkey</t>
-  </si>
-  <si>
     <t>North Macedonia</t>
   </si>
   <si>
@@ -355,6 +352,9 @@
   </si>
   <si>
     <t>Tunisia</t>
+  </si>
+  <si>
+    <t>Türkiye, Republic of</t>
   </si>
 </sst>
 </file>
@@ -1222,14 +1222,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z78"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="31.81640625" customWidth="1"/>
-    <col min="2" max="2" width="24.26953125" customWidth="1"/>
-    <col min="3" max="3" width="7.08984375" customWidth="1"/>
+    <col min="1" max="1" width="31.85546875" customWidth="1"/>
+    <col min="2" max="2" width="24.28515625" customWidth="1"/>
+    <col min="3" max="3" width="7.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1240,19 +1240,19 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>33</v>
       </c>
       <c r="B2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C2" s="3">
         <v>2025</v>
       </c>
       <c r="Z2" s="1"/>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>34</v>
       </c>
@@ -1264,7 +1264,7 @@
       </c>
       <c r="Z3" s="1"/>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>35</v>
       </c>
@@ -1276,19 +1276,19 @@
       </c>
       <c r="Z4" s="1"/>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>36</v>
       </c>
       <c r="B5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C5" s="3">
         <v>2025</v>
       </c>
       <c r="Z5" s="1"/>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>37</v>
       </c>
@@ -1300,7 +1300,7 @@
       </c>
       <c r="Z6" s="1"/>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>38</v>
       </c>
@@ -1312,7 +1312,7 @@
       </c>
       <c r="Z7" s="1"/>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>39</v>
       </c>
@@ -1324,31 +1324,31 @@
       </c>
       <c r="Z8" s="1"/>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>40</v>
       </c>
       <c r="B9" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C9" s="3">
         <v>2025</v>
       </c>
       <c r="Z9" s="1"/>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>41</v>
       </c>
       <c r="B10" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C10" s="3">
         <v>2025</v>
       </c>
       <c r="Z10" s="1"/>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>42</v>
       </c>
@@ -1360,7 +1360,7 @@
       </c>
       <c r="Z11" s="1"/>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>43</v>
       </c>
@@ -1372,31 +1372,31 @@
       </c>
       <c r="Z12" s="1"/>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>44</v>
       </c>
       <c r="B13" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C13" s="3">
         <v>2025</v>
       </c>
       <c r="Z13" s="1"/>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>45</v>
       </c>
       <c r="B14" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C14" s="3">
         <v>2025</v>
       </c>
       <c r="Z14" s="1"/>
     </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>46</v>
       </c>
@@ -1408,7 +1408,7 @@
       </c>
       <c r="Z15" s="1"/>
     </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>47</v>
       </c>
@@ -1420,7 +1420,7 @@
       </c>
       <c r="Z16" s="1"/>
     </row>
-    <row r="17" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>48</v>
       </c>
@@ -1432,19 +1432,19 @@
       </c>
       <c r="Z17" s="1"/>
     </row>
-    <row r="18" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>49</v>
       </c>
       <c r="B18" t="s">
-        <v>95</v>
+        <v>109</v>
       </c>
       <c r="C18" s="3">
         <v>2025</v>
       </c>
       <c r="Z18" s="1"/>
     </row>
-    <row r="19" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>50</v>
       </c>
@@ -1456,7 +1456,7 @@
       </c>
       <c r="Z19" s="1"/>
     </row>
-    <row r="20" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>51</v>
       </c>
@@ -1468,7 +1468,7 @@
       </c>
       <c r="Z20" s="1"/>
     </row>
-    <row r="21" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>52</v>
       </c>
@@ -1480,7 +1480,7 @@
       </c>
       <c r="Z21" s="1"/>
     </row>
-    <row r="22" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>53</v>
       </c>
@@ -1492,19 +1492,19 @@
       </c>
       <c r="Z22" s="1"/>
     </row>
-    <row r="23" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>54</v>
       </c>
       <c r="B23" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C23" s="3">
         <v>2025</v>
       </c>
       <c r="Z23" s="1"/>
     </row>
-    <row r="24" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>55</v>
       </c>
@@ -1516,19 +1516,19 @@
       </c>
       <c r="Z24" s="1"/>
     </row>
-    <row r="25" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>56</v>
       </c>
       <c r="B25" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C25" s="3">
         <v>2025</v>
       </c>
       <c r="Z25" s="1"/>
     </row>
-    <row r="26" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>57</v>
       </c>
@@ -1540,19 +1540,19 @@
       </c>
       <c r="Z26" s="1"/>
     </row>
-    <row r="27" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>58</v>
       </c>
       <c r="B27" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C27" s="3">
         <v>2025</v>
       </c>
       <c r="Z27" s="1"/>
     </row>
-    <row r="28" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>59</v>
       </c>
@@ -1564,19 +1564,19 @@
       </c>
       <c r="Z28" s="1"/>
     </row>
-    <row r="29" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>60</v>
       </c>
       <c r="B29" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C29" s="3">
         <v>2025</v>
       </c>
       <c r="Z29" s="1"/>
     </row>
-    <row r="30" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>61</v>
       </c>
@@ -1588,7 +1588,7 @@
       </c>
       <c r="Z30" s="1"/>
     </row>
-    <row r="31" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>62</v>
       </c>
@@ -1600,19 +1600,19 @@
       </c>
       <c r="Z31" s="1"/>
     </row>
-    <row r="32" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>63</v>
       </c>
       <c r="B32" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C32" s="3">
         <v>2025</v>
       </c>
       <c r="Z32" s="1"/>
     </row>
-    <row r="33" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>64</v>
       </c>
@@ -1624,19 +1624,19 @@
       </c>
       <c r="Z33" s="1"/>
     </row>
-    <row r="34" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>65</v>
       </c>
       <c r="B34" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C34" s="3">
         <v>2025</v>
       </c>
       <c r="Z34" s="1"/>
     </row>
-    <row r="35" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>66</v>
       </c>
@@ -1648,19 +1648,19 @@
       </c>
       <c r="Z35" s="1"/>
     </row>
-    <row r="36" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>67</v>
       </c>
       <c r="B36" t="s">
-        <v>95</v>
+        <v>109</v>
       </c>
       <c r="C36" s="3">
         <v>2025</v>
       </c>
       <c r="Z36" s="1"/>
     </row>
-    <row r="37" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>68</v>
       </c>
@@ -1672,31 +1672,31 @@
       </c>
       <c r="Z37" s="1"/>
     </row>
-    <row r="38" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>69</v>
       </c>
       <c r="B38" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C38" s="3">
         <v>2025</v>
       </c>
       <c r="Z38" s="1"/>
     </row>
-    <row r="39" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>70</v>
       </c>
       <c r="B39" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C39" s="3">
         <v>2025</v>
       </c>
       <c r="Z39" s="1"/>
     </row>
-    <row r="40" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>71</v>
       </c>
@@ -1708,19 +1708,19 @@
       </c>
       <c r="Z40" s="1"/>
     </row>
-    <row r="41" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>72</v>
       </c>
       <c r="B41" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C41" s="3">
         <v>2025</v>
       </c>
       <c r="Z41" s="1"/>
     </row>
-    <row r="42" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>73</v>
       </c>
@@ -1732,31 +1732,31 @@
       </c>
       <c r="Z42" s="1"/>
     </row>
-    <row r="43" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>74</v>
       </c>
       <c r="B43" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C43" s="3">
         <v>2025</v>
       </c>
       <c r="Z43" s="1"/>
     </row>
-    <row r="44" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>75</v>
       </c>
       <c r="B44" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C44" s="3">
         <v>2025</v>
       </c>
       <c r="Z44" s="1"/>
     </row>
-    <row r="45" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>76</v>
       </c>
@@ -1768,7 +1768,7 @@
       </c>
       <c r="Z45" s="1"/>
     </row>
-    <row r="46" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>77</v>
       </c>
@@ -1780,7 +1780,7 @@
       </c>
       <c r="Z46" s="1"/>
     </row>
-    <row r="47" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>78</v>
       </c>
@@ -1792,19 +1792,19 @@
       </c>
       <c r="Z47" s="1"/>
     </row>
-    <row r="48" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>79</v>
       </c>
       <c r="B48" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C48" s="3">
         <v>2025</v>
       </c>
       <c r="Z48" s="1"/>
     </row>
-    <row r="49" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>3</v>
       </c>
@@ -1816,7 +1816,7 @@
       </c>
       <c r="Z49" s="1"/>
     </row>
-    <row r="50" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>4</v>
       </c>
@@ -1828,7 +1828,7 @@
       </c>
       <c r="Z50" s="1"/>
     </row>
-    <row r="51" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>5</v>
       </c>
@@ -1840,7 +1840,7 @@
       </c>
       <c r="Z51" s="1"/>
     </row>
-    <row r="52" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>6</v>
       </c>
@@ -1852,7 +1852,7 @@
       </c>
       <c r="Z52" s="1"/>
     </row>
-    <row r="53" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>7</v>
       </c>
@@ -1864,7 +1864,7 @@
       </c>
       <c r="Z53" s="1"/>
     </row>
-    <row r="54" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>8</v>
       </c>
@@ -1876,7 +1876,7 @@
       </c>
       <c r="Z54" s="1"/>
     </row>
-    <row r="55" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>9</v>
       </c>
@@ -1888,7 +1888,7 @@
       </c>
       <c r="Z55" s="1"/>
     </row>
-    <row r="56" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>10</v>
       </c>
@@ -1900,7 +1900,7 @@
       </c>
       <c r="Z56" s="1"/>
     </row>
-    <row r="57" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>11</v>
       </c>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="Z57" s="1"/>
     </row>
-    <row r="58" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>12</v>
       </c>
@@ -1924,7 +1924,7 @@
       </c>
       <c r="Z58" s="1"/>
     </row>
-    <row r="59" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>13</v>
       </c>
@@ -1936,7 +1936,7 @@
       </c>
       <c r="Z59" s="1"/>
     </row>
-    <row r="60" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>14</v>
       </c>
@@ -1948,7 +1948,7 @@
       </c>
       <c r="Z60" s="1"/>
     </row>
-    <row r="61" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>15</v>
       </c>
@@ -1961,7 +1961,7 @@
       <c r="E61" s="2"/>
       <c r="Z61" s="1"/>
     </row>
-    <row r="62" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>16</v>
       </c>
@@ -1973,7 +1973,7 @@
       </c>
       <c r="Z62" s="1"/>
     </row>
-    <row r="63" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>17</v>
       </c>
@@ -1985,7 +1985,7 @@
       </c>
       <c r="Z63" s="1"/>
     </row>
-    <row r="64" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>18</v>
       </c>
@@ -1997,7 +1997,7 @@
       </c>
       <c r="Z64" s="1"/>
     </row>
-    <row r="65" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>19</v>
       </c>
@@ -2009,7 +2009,7 @@
       </c>
       <c r="Z65" s="1"/>
     </row>
-    <row r="66" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>20</v>
       </c>
@@ -2021,7 +2021,7 @@
       </c>
       <c r="Z66" s="1"/>
     </row>
-    <row r="67" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>21</v>
       </c>
@@ -2033,7 +2033,7 @@
       </c>
       <c r="Z67" s="1"/>
     </row>
-    <row r="68" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>22</v>
       </c>
@@ -2045,7 +2045,7 @@
       </c>
       <c r="Z68" s="1"/>
     </row>
-    <row r="69" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>23</v>
       </c>
@@ -2057,7 +2057,7 @@
       </c>
       <c r="Z69" s="1"/>
     </row>
-    <row r="70" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>24</v>
       </c>
@@ -2069,7 +2069,7 @@
       </c>
       <c r="Z70" s="1"/>
     </row>
-    <row r="71" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>25</v>
       </c>
@@ -2081,7 +2081,7 @@
       </c>
       <c r="Z71" s="1"/>
     </row>
-    <row r="72" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>26</v>
       </c>
@@ -2093,7 +2093,7 @@
       </c>
       <c r="Z72" s="1"/>
     </row>
-    <row r="73" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>27</v>
       </c>
@@ -2105,7 +2105,7 @@
       </c>
       <c r="Z73" s="1"/>
     </row>
-    <row r="74" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>28</v>
       </c>
@@ -2117,7 +2117,7 @@
       </c>
       <c r="Z74" s="1"/>
     </row>
-    <row r="75" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>29</v>
       </c>
@@ -2129,7 +2129,7 @@
       </c>
       <c r="Z75" s="1"/>
     </row>
-    <row r="76" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>30</v>
       </c>
@@ -2141,7 +2141,7 @@
       </c>
       <c r="Z76" s="1"/>
     </row>
-    <row r="77" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>31</v>
       </c>
@@ -2152,12 +2152,12 @@
         <v>2024</v>
       </c>
     </row>
-    <row r="78" spans="1:26" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>32</v>
       </c>
       <c r="B78" t="s">
-        <v>95</v>
+        <v>109</v>
       </c>
       <c r="C78" s="3">
         <v>2024</v>

</xml_diff>

<commit_message>
Cross-hatching pattern added for regional only countries
</commit_message>
<xml_diff>
--- a/data/GTF BIG Talent Scholars.xlsx
+++ b/data/GTF BIG Talent Scholars.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\iona.sms.ed.ac.uk\home\s2730428\GTF-Impact-Map\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\s2730428\Documents\GTF-Impact-Map\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{044BD7FC-82BE-4106-904E-83837A500776}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3821E74-08AC-462B-BB68-1C28E9D85A9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="1190" windowWidth="14400" windowHeight="7270" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Global Talent Fund - BIG Schola" sheetId="1" r:id="rId1"/>
@@ -288,9 +288,6 @@
     <t>Germany</t>
   </si>
   <si>
-    <t>Hong Kong, China</t>
-  </si>
-  <si>
     <t>Brazil</t>
   </si>
   <si>
@@ -355,6 +352,9 @@
   </si>
   <si>
     <t>Türkiye, Republic of</t>
+  </si>
+  <si>
+    <t>Hong Kong SAR</t>
   </si>
 </sst>
 </file>
@@ -1222,14 +1222,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z78"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="31.85546875" customWidth="1"/>
-    <col min="2" max="2" width="24.28515625" customWidth="1"/>
-    <col min="3" max="3" width="7.140625" customWidth="1"/>
+    <col min="1" max="1" width="31.81640625" customWidth="1"/>
+    <col min="2" max="2" width="24.26953125" customWidth="1"/>
+    <col min="3" max="3" width="7.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1240,19 +1240,19 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>33</v>
       </c>
       <c r="B2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C2" s="3">
         <v>2025</v>
       </c>
       <c r="Z2" s="1"/>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>34</v>
       </c>
@@ -1264,31 +1264,31 @@
       </c>
       <c r="Z3" s="1"/>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>35</v>
       </c>
       <c r="B4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C4" s="3">
         <v>2025</v>
       </c>
       <c r="Z4" s="1"/>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>36</v>
       </c>
       <c r="B5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C5" s="3">
         <v>2025</v>
       </c>
       <c r="Z5" s="1"/>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>37</v>
       </c>
@@ -1300,7 +1300,7 @@
       </c>
       <c r="Z6" s="1"/>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>38</v>
       </c>
@@ -1312,7 +1312,7 @@
       </c>
       <c r="Z7" s="1"/>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>39</v>
       </c>
@@ -1324,79 +1324,79 @@
       </c>
       <c r="Z8" s="1"/>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>40</v>
       </c>
       <c r="B9" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C9" s="3">
         <v>2025</v>
       </c>
       <c r="Z9" s="1"/>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>41</v>
       </c>
       <c r="B10" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C10" s="3">
         <v>2025</v>
       </c>
       <c r="Z10" s="1"/>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>42</v>
       </c>
       <c r="B11" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C11" s="3">
         <v>2025</v>
       </c>
       <c r="Z11" s="1"/>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>43</v>
       </c>
       <c r="B12" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C12" s="3">
         <v>2025</v>
       </c>
       <c r="Z12" s="1"/>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>44</v>
       </c>
       <c r="B13" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C13" s="3">
         <v>2025</v>
       </c>
       <c r="Z13" s="1"/>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>45</v>
       </c>
       <c r="B14" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C14" s="3">
         <v>2025</v>
       </c>
       <c r="Z14" s="1"/>
     </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>46</v>
       </c>
@@ -1408,19 +1408,19 @@
       </c>
       <c r="Z15" s="1"/>
     </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>47</v>
       </c>
       <c r="B16" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C16" s="3">
         <v>2025</v>
       </c>
       <c r="Z16" s="1"/>
     </row>
-    <row r="17" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>48</v>
       </c>
@@ -1432,19 +1432,19 @@
       </c>
       <c r="Z17" s="1"/>
     </row>
-    <row r="18" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>49</v>
       </c>
       <c r="B18" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C18" s="3">
         <v>2025</v>
       </c>
       <c r="Z18" s="1"/>
     </row>
-    <row r="19" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>50</v>
       </c>
@@ -1456,31 +1456,31 @@
       </c>
       <c r="Z19" s="1"/>
     </row>
-    <row r="20" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>51</v>
       </c>
       <c r="B20" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C20" s="3">
         <v>2025</v>
       </c>
       <c r="Z20" s="1"/>
     </row>
-    <row r="21" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>52</v>
       </c>
       <c r="B21" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C21" s="3">
         <v>2025</v>
       </c>
       <c r="Z21" s="1"/>
     </row>
-    <row r="22" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>53</v>
       </c>
@@ -1492,67 +1492,67 @@
       </c>
       <c r="Z22" s="1"/>
     </row>
-    <row r="23" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>54</v>
       </c>
       <c r="B23" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C23" s="3">
         <v>2025</v>
       </c>
       <c r="Z23" s="1"/>
     </row>
-    <row r="24" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>55</v>
       </c>
       <c r="B24" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C24" s="3">
         <v>2025</v>
       </c>
       <c r="Z24" s="1"/>
     </row>
-    <row r="25" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>56</v>
       </c>
       <c r="B25" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C25" s="3">
         <v>2025</v>
       </c>
       <c r="Z25" s="1"/>
     </row>
-    <row r="26" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>57</v>
       </c>
       <c r="B26" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C26" s="3">
         <v>2025</v>
       </c>
       <c r="Z26" s="1"/>
     </row>
-    <row r="27" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>58</v>
       </c>
       <c r="B27" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C27" s="3">
         <v>2025</v>
       </c>
       <c r="Z27" s="1"/>
     </row>
-    <row r="28" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>59</v>
       </c>
@@ -1564,19 +1564,19 @@
       </c>
       <c r="Z28" s="1"/>
     </row>
-    <row r="29" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>60</v>
       </c>
       <c r="B29" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C29" s="3">
         <v>2025</v>
       </c>
       <c r="Z29" s="1"/>
     </row>
-    <row r="30" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>61</v>
       </c>
@@ -1588,55 +1588,55 @@
       </c>
       <c r="Z30" s="1"/>
     </row>
-    <row r="31" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>62</v>
       </c>
       <c r="B31" t="s">
-        <v>87</v>
+        <v>109</v>
       </c>
       <c r="C31" s="3">
         <v>2025</v>
       </c>
       <c r="Z31" s="1"/>
     </row>
-    <row r="32" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>63</v>
       </c>
       <c r="B32" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C32" s="3">
         <v>2025</v>
       </c>
       <c r="Z32" s="1"/>
     </row>
-    <row r="33" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>64</v>
       </c>
       <c r="B33" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C33" s="3">
         <v>2025</v>
       </c>
       <c r="Z33" s="1"/>
     </row>
-    <row r="34" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>65</v>
       </c>
       <c r="B34" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C34" s="3">
         <v>2025</v>
       </c>
       <c r="Z34" s="1"/>
     </row>
-    <row r="35" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>66</v>
       </c>
@@ -1648,79 +1648,79 @@
       </c>
       <c r="Z35" s="1"/>
     </row>
-    <row r="36" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>67</v>
       </c>
       <c r="B36" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C36" s="3">
         <v>2025</v>
       </c>
       <c r="Z36" s="1"/>
     </row>
-    <row r="37" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>68</v>
       </c>
       <c r="B37" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C37" s="3">
         <v>2025</v>
       </c>
       <c r="Z37" s="1"/>
     </row>
-    <row r="38" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>69</v>
       </c>
       <c r="B38" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C38" s="3">
         <v>2025</v>
       </c>
       <c r="Z38" s="1"/>
     </row>
-    <row r="39" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>70</v>
       </c>
       <c r="B39" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C39" s="3">
         <v>2025</v>
       </c>
       <c r="Z39" s="1"/>
     </row>
-    <row r="40" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>71</v>
       </c>
       <c r="B40" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C40" s="3">
         <v>2025</v>
       </c>
       <c r="Z40" s="1"/>
     </row>
-    <row r="41" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>72</v>
       </c>
       <c r="B41" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C41" s="3">
         <v>2025</v>
       </c>
       <c r="Z41" s="1"/>
     </row>
-    <row r="42" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>73</v>
       </c>
@@ -1732,79 +1732,79 @@
       </c>
       <c r="Z42" s="1"/>
     </row>
-    <row r="43" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>74</v>
       </c>
       <c r="B43" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C43" s="3">
         <v>2025</v>
       </c>
       <c r="Z43" s="1"/>
     </row>
-    <row r="44" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>75</v>
       </c>
       <c r="B44" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C44" s="3">
         <v>2025</v>
       </c>
       <c r="Z44" s="1"/>
     </row>
-    <row r="45" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>76</v>
       </c>
       <c r="B45" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C45" s="3">
         <v>2025</v>
       </c>
       <c r="Z45" s="1"/>
     </row>
-    <row r="46" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>77</v>
       </c>
       <c r="B46" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C46" s="3">
         <v>2025</v>
       </c>
       <c r="Z46" s="1"/>
     </row>
-    <row r="47" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>78</v>
       </c>
       <c r="B47" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C47" s="3">
         <v>2025</v>
       </c>
       <c r="Z47" s="1"/>
     </row>
-    <row r="48" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>79</v>
       </c>
       <c r="B48" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C48" s="3">
         <v>2025</v>
       </c>
       <c r="Z48" s="1"/>
     </row>
-    <row r="49" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>3</v>
       </c>
@@ -1816,7 +1816,7 @@
       </c>
       <c r="Z49" s="1"/>
     </row>
-    <row r="50" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>4</v>
       </c>
@@ -1828,7 +1828,7 @@
       </c>
       <c r="Z50" s="1"/>
     </row>
-    <row r="51" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>5</v>
       </c>
@@ -1840,7 +1840,7 @@
       </c>
       <c r="Z51" s="1"/>
     </row>
-    <row r="52" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>6</v>
       </c>
@@ -1852,7 +1852,7 @@
       </c>
       <c r="Z52" s="1"/>
     </row>
-    <row r="53" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>7</v>
       </c>
@@ -1864,7 +1864,7 @@
       </c>
       <c r="Z53" s="1"/>
     </row>
-    <row r="54" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>8</v>
       </c>
@@ -1876,7 +1876,7 @@
       </c>
       <c r="Z54" s="1"/>
     </row>
-    <row r="55" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>9</v>
       </c>
@@ -1888,7 +1888,7 @@
       </c>
       <c r="Z55" s="1"/>
     </row>
-    <row r="56" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>10</v>
       </c>
@@ -1900,7 +1900,7 @@
       </c>
       <c r="Z56" s="1"/>
     </row>
-    <row r="57" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>11</v>
       </c>
@@ -1912,7 +1912,7 @@
       </c>
       <c r="Z57" s="1"/>
     </row>
-    <row r="58" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>12</v>
       </c>
@@ -1924,7 +1924,7 @@
       </c>
       <c r="Z58" s="1"/>
     </row>
-    <row r="59" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>13</v>
       </c>
@@ -1936,7 +1936,7 @@
       </c>
       <c r="Z59" s="1"/>
     </row>
-    <row r="60" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>14</v>
       </c>
@@ -1948,7 +1948,7 @@
       </c>
       <c r="Z60" s="1"/>
     </row>
-    <row r="61" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>15</v>
       </c>
@@ -1961,7 +1961,7 @@
       <c r="E61" s="2"/>
       <c r="Z61" s="1"/>
     </row>
-    <row r="62" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>16</v>
       </c>
@@ -1973,7 +1973,7 @@
       </c>
       <c r="Z62" s="1"/>
     </row>
-    <row r="63" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>17</v>
       </c>
@@ -1985,7 +1985,7 @@
       </c>
       <c r="Z63" s="1"/>
     </row>
-    <row r="64" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>18</v>
       </c>
@@ -1997,7 +1997,7 @@
       </c>
       <c r="Z64" s="1"/>
     </row>
-    <row r="65" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>19</v>
       </c>
@@ -2009,7 +2009,7 @@
       </c>
       <c r="Z65" s="1"/>
     </row>
-    <row r="66" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>20</v>
       </c>
@@ -2021,7 +2021,7 @@
       </c>
       <c r="Z66" s="1"/>
     </row>
-    <row r="67" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>21</v>
       </c>
@@ -2033,7 +2033,7 @@
       </c>
       <c r="Z67" s="1"/>
     </row>
-    <row r="68" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>22</v>
       </c>
@@ -2045,119 +2045,119 @@
       </c>
       <c r="Z68" s="1"/>
     </row>
-    <row r="69" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>23</v>
       </c>
       <c r="B69" t="s">
-        <v>87</v>
+        <v>109</v>
       </c>
       <c r="C69" s="3">
         <v>2024</v>
       </c>
       <c r="Z69" s="1"/>
     </row>
-    <row r="70" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>24</v>
       </c>
       <c r="B70" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C70" s="3">
         <v>2024</v>
       </c>
       <c r="Z70" s="1"/>
     </row>
-    <row r="71" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>25</v>
       </c>
       <c r="B71" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C71" s="3">
         <v>2024</v>
       </c>
       <c r="Z71" s="1"/>
     </row>
-    <row r="72" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>26</v>
       </c>
       <c r="B72" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C72" s="3">
         <v>2024</v>
       </c>
       <c r="Z72" s="1"/>
     </row>
-    <row r="73" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>27</v>
       </c>
       <c r="B73" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C73" s="3">
         <v>2024</v>
       </c>
       <c r="Z73" s="1"/>
     </row>
-    <row r="74" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>28</v>
       </c>
       <c r="B74" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C74" s="3">
         <v>2024</v>
       </c>
       <c r="Z74" s="1"/>
     </row>
-    <row r="75" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>29</v>
       </c>
       <c r="B75" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C75" s="3">
         <v>2024</v>
       </c>
       <c r="Z75" s="1"/>
     </row>
-    <row r="76" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>30</v>
       </c>
       <c r="B76" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C76" s="3">
         <v>2024</v>
       </c>
       <c r="Z76" s="1"/>
     </row>
-    <row r="77" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>31</v>
       </c>
       <c r="B77" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C77" s="3">
         <v>2024</v>
       </c>
     </row>
-    <row r="78" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>32</v>
       </c>
       <c r="B78" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C78" s="3">
         <v>2024</v>

</xml_diff>